<commit_message>
Simplify B4 HIREF workbook contract
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/src/sample-data/excel/team_project_capacity_workbook_hiref_sample.xlsx
+++ b/src/sample-data/excel/team_project_capacity_workbook_hiref_sample.xlsx
@@ -12,10 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Allocations" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capacity" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIREF Members" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIREF Slots" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIREF Placeholders" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIREF Placeholder Allocations" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIREF Requests" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,6 +530,11 @@
           <t>effective_end</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>next_hiref_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -619,6 +621,46 @@
         <v>7</v>
       </c>
       <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>HIREF-SYNTH-CEDAR-NEXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>member-synthetic-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Casey Example</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>LTFTE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
@@ -771,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,6 +837,11 @@
           <t>allocation</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>hiref_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -874,6 +921,26 @@
       </c>
       <c r="D5" t="n">
         <v>0.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>project-synthetic-beacon</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HIREF-SYNTH-OPEN-001</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -887,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -998,6 +1065,48 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>member-synthetic-003</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>member-synthetic-003</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1012,44 +1121,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>member_key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>next_hiref_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>member-synthetic-002</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>HIREF-SYNTH-CEDAR-NEXT</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1061,7 +1132,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>project_key</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1093,7 +1164,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Project Atlas (project-synthetic-atlas)</t>
+          <t>project-synthetic-atlas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1111,7 +1182,11 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SYNTHETIC_DATASET_V1 current contract slot</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1121,7 +1196,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Project Cedar (project-synthetic-cedar)</t>
+          <t>project-synthetic-cedar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1139,7 +1214,6 @@
           <t>2026-10-31</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1149,7 +1223,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Project Cedar (project-synthetic-cedar)</t>
+          <t>project-synthetic-cedar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1181,7 +1255,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Project Beacon (project-synthetic-beacon)</t>
+          <t>project-synthetic-beacon</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1201,148 +1275,8 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open contractor demand SYNTHETIC_DATASET_V1</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>placeholder_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>display_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>hiref_id</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>linked_member_key</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>resource_type</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>placeholder-synthetic-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>To Be Hired</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>HIREF-SYNTH-OPEN-001</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>STFTE</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
           <t>Open contractor demand</t>
         </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>placeholder_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>project_key</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>allocation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>placeholder-synthetic-001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>project-synthetic-beacon</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>